<commit_message>
Fix zeros in monthly resolution table on macOS Excel
The monthly table read from formula-only helper columns that macOS Excel
did not recalculate, so every value showed 0. Write the Datos resolution
(hours, days, month) columns as concrete values and set fullCalcOnLoad so
the summary formulas recompute on open.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nn9QKEstPX9eZ4ngSPWHBW
</commit_message>
<xml_diff>
--- a/Portal_Uploads_Metricas.xlsx
+++ b/Portal_Uploads_Metricas.xlsx
@@ -9910,17 +9910,12 @@
         <v>46013.89421296296</v>
       </c>
       <c r="E2" s="18" t="n"/>
-      <c r="F2" s="9">
-        <f>IF(OR(D2="",E2=""),"",(E2-D2)*24)</f>
-        <v/>
-      </c>
-      <c r="G2" s="9">
-        <f>IF(F2="","",F2/24)</f>
-        <v/>
-      </c>
-      <c r="H2" s="19">
-        <f>IF(D2="","",TEXT(D2,"YYYY-MM"))</f>
-        <v/>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="19" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -9945,17 +9940,16 @@
       <c r="E3" s="18" t="n">
         <v>46176.46725694444</v>
       </c>
-      <c r="F3" s="9">
-        <f>IF(OR(D3="",E3=""),"",(E3-D3)*24)</f>
-        <v/>
-      </c>
-      <c r="G3" s="9">
-        <f>IF(F3="","",F3/24)</f>
-        <v/>
-      </c>
-      <c r="H3" s="19">
-        <f>IF(D3="","",TEXT(D3,"YYYY-MM"))</f>
-        <v/>
+      <c r="F3" s="9" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H3" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -9980,17 +9974,16 @@
       <c r="E4" s="18" t="n">
         <v>46176.56564814815</v>
       </c>
-      <c r="F4" s="9">
-        <f>IF(OR(D4="",E4=""),"",(E4-D4)*24)</f>
-        <v/>
-      </c>
-      <c r="G4" s="9">
-        <f>IF(F4="","",F4/24)</f>
-        <v/>
-      </c>
-      <c r="H4" s="19">
-        <f>IF(D4="","",TEXT(D4,"YYYY-MM"))</f>
-        <v/>
+      <c r="F4" s="9" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -10015,17 +10008,16 @@
       <c r="E5" s="18" t="n">
         <v>46177.52550925926</v>
       </c>
-      <c r="F5" s="9">
-        <f>IF(OR(D5="",E5=""),"",(E5-D5)*24)</f>
-        <v/>
-      </c>
-      <c r="G5" s="9">
-        <f>IF(F5="","",F5/24)</f>
-        <v/>
-      </c>
-      <c r="H5" s="19">
-        <f>IF(D5="","",TEXT(D5,"YYYY-MM"))</f>
-        <v/>
+      <c r="F5" s="9" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -10050,17 +10042,16 @@
       <c r="E6" s="18" t="n">
         <v>46177.51328703704</v>
       </c>
-      <c r="F6" s="9">
-        <f>IF(OR(D6="",E6=""),"",(E6-D6)*24)</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
-        <f>IF(F6="","",F6/24)</f>
-        <v/>
-      </c>
-      <c r="H6" s="19">
-        <f>IF(D6="","",TEXT(D6,"YYYY-MM"))</f>
-        <v/>
+      <c r="F6" s="9" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -10085,17 +10076,16 @@
       <c r="E7" s="18" t="n">
         <v>46178.41920138889</v>
       </c>
-      <c r="F7" s="9">
-        <f>IF(OR(D7="",E7=""),"",(E7-D7)*24)</f>
-        <v/>
-      </c>
-      <c r="G7" s="9">
-        <f>IF(F7="","",F7/24)</f>
-        <v/>
-      </c>
-      <c r="H7" s="19">
-        <f>IF(D7="","",TEXT(D7,"YYYY-MM"))</f>
-        <v/>
+      <c r="F7" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -10120,17 +10110,16 @@
       <c r="E8" s="18" t="n">
         <v>46197.53972222222</v>
       </c>
-      <c r="F8" s="9">
-        <f>IF(OR(D8="",E8=""),"",(E8-D8)*24)</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
-        <f>IF(F8="","",F8/24)</f>
-        <v/>
-      </c>
-      <c r="H8" s="19">
-        <f>IF(D8="","",TEXT(D8,"YYYY-MM"))</f>
-        <v/>
+      <c r="F8" s="9" t="n">
+        <v>470.1</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -10155,17 +10144,16 @@
       <c r="E9" s="18" t="n">
         <v>46178.56423611111</v>
       </c>
-      <c r="F9" s="9">
-        <f>IF(OR(D9="",E9=""),"",(E9-D9)*24)</f>
-        <v/>
-      </c>
-      <c r="G9" s="9">
-        <f>IF(F9="","",F9/24)</f>
-        <v/>
-      </c>
-      <c r="H9" s="19">
-        <f>IF(D9="","",TEXT(D9,"YYYY-MM"))</f>
-        <v/>
+      <c r="F9" s="9" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -10186,17 +10174,16 @@
       <c r="E10" s="18" t="n">
         <v>46178.60672453704</v>
       </c>
-      <c r="F10" s="9">
-        <f>IF(OR(D10="",E10=""),"",(E10-D10)*24)</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
-        <f>IF(F10="","",F10/24)</f>
-        <v/>
-      </c>
-      <c r="H10" s="19">
-        <f>IF(D10="","",TEXT(D10,"YYYY-MM"))</f>
-        <v/>
+      <c r="F10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -10221,17 +10208,16 @@
       <c r="E11" s="18" t="n">
         <v>46183.64862268518</v>
       </c>
-      <c r="F11" s="9">
-        <f>IF(OR(D11="",E11=""),"",(E11-D11)*24)</f>
-        <v/>
-      </c>
-      <c r="G11" s="9">
-        <f>IF(F11="","",F11/24)</f>
-        <v/>
-      </c>
-      <c r="H11" s="19">
-        <f>IF(D11="","",TEXT(D11,"YYYY-MM"))</f>
-        <v/>
+      <c r="F11" s="9" t="n">
+        <v>121.5</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -10256,17 +10242,16 @@
       <c r="E12" s="18" t="n">
         <v>46182.33144675926</v>
       </c>
-      <c r="F12" s="9">
-        <f>IF(OR(D12="",E12=""),"",(E12-D12)*24)</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
-        <f>IF(F12="","",F12/24)</f>
-        <v/>
-      </c>
-      <c r="H12" s="19">
-        <f>IF(D12="","",TEXT(D12,"YYYY-MM"))</f>
-        <v/>
+      <c r="F12" s="9" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -10291,17 +10276,16 @@
       <c r="E13" s="18" t="n">
         <v>46183.6115162037</v>
       </c>
-      <c r="F13" s="9">
-        <f>IF(OR(D13="",E13=""),"",(E13-D13)*24)</f>
-        <v/>
-      </c>
-      <c r="G13" s="9">
-        <f>IF(F13="","",F13/24)</f>
-        <v/>
-      </c>
-      <c r="H13" s="19">
-        <f>IF(D13="","",TEXT(D13,"YYYY-MM"))</f>
-        <v/>
+      <c r="F13" s="9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -10326,17 +10310,16 @@
       <c r="E14" s="18" t="n">
         <v>46197.54549768518</v>
       </c>
-      <c r="F14" s="9">
-        <f>IF(OR(D14="",E14=""),"",(E14-D14)*24)</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
-        <f>IF(F14="","",F14/24)</f>
-        <v/>
-      </c>
-      <c r="H14" s="19">
-        <f>IF(D14="","",TEXT(D14,"YYYY-MM"))</f>
-        <v/>
+      <c r="F14" s="9" t="n">
+        <v>332.7</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -10361,17 +10344,16 @@
       <c r="E15" s="18" t="n">
         <v>46185.421875</v>
       </c>
-      <c r="F15" s="9">
-        <f>IF(OR(D15="",E15=""),"",(E15-D15)*24)</f>
-        <v/>
-      </c>
-      <c r="G15" s="9">
-        <f>IF(F15="","",F15/24)</f>
-        <v/>
-      </c>
-      <c r="H15" s="19">
-        <f>IF(D15="","",TEXT(D15,"YYYY-MM"))</f>
-        <v/>
+      <c r="F15" s="9" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -10396,17 +10378,16 @@
       <c r="E16" s="18" t="n">
         <v>46185.48872685185</v>
       </c>
-      <c r="F16" s="9">
-        <f>IF(OR(D16="",E16=""),"",(E16-D16)*24)</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
-        <f>IF(F16="","",F16/24)</f>
-        <v/>
-      </c>
-      <c r="H16" s="19">
-        <f>IF(D16="","",TEXT(D16,"YYYY-MM"))</f>
-        <v/>
+      <c r="F16" s="9" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -10431,17 +10412,16 @@
       <c r="E17" s="18" t="n">
         <v>46197.5468287037</v>
       </c>
-      <c r="F17" s="9">
-        <f>IF(OR(D17="",E17=""),"",(E17-D17)*24)</f>
-        <v/>
-      </c>
-      <c r="G17" s="9">
-        <f>IF(F17="","",F17/24)</f>
-        <v/>
-      </c>
-      <c r="H17" s="19">
-        <f>IF(D17="","",TEXT(D17,"YYYY-MM"))</f>
-        <v/>
+      <c r="F17" s="9" t="n">
+        <v>288.7</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -10466,17 +10446,16 @@
       <c r="E18" s="18" t="n">
         <v>46192.57513888889</v>
       </c>
-      <c r="F18" s="9">
-        <f>IF(OR(D18="",E18=""),"",(E18-D18)*24)</f>
-        <v/>
-      </c>
-      <c r="G18" s="9">
-        <f>IF(F18="","",F18/24)</f>
-        <v/>
-      </c>
-      <c r="H18" s="19">
-        <f>IF(D18="","",TEXT(D18,"YYYY-MM"))</f>
-        <v/>
+      <c r="F18" s="9" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -10501,17 +10480,16 @@
       <c r="E19" s="18" t="n">
         <v>46197.55075231481</v>
       </c>
-      <c r="F19" s="9">
-        <f>IF(OR(D19="",E19=""),"",(E19-D19)*24)</f>
-        <v/>
-      </c>
-      <c r="G19" s="9">
-        <f>IF(F19="","",F19/24)</f>
-        <v/>
-      </c>
-      <c r="H19" s="19">
-        <f>IF(D19="","",TEXT(D19,"YYYY-MM"))</f>
-        <v/>
+      <c r="F19" s="9" t="n">
+        <v>218.8</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -10536,17 +10514,16 @@
       <c r="E20" s="18" t="n">
         <v>46189.31497685185</v>
       </c>
-      <c r="F20" s="9">
-        <f>IF(OR(D20="",E20=""),"",(E20-D20)*24)</f>
-        <v/>
-      </c>
-      <c r="G20" s="9">
-        <f>IF(F20="","",F20/24)</f>
-        <v/>
-      </c>
-      <c r="H20" s="19">
-        <f>IF(D20="","",TEXT(D20,"YYYY-MM"))</f>
-        <v/>
+      <c r="F20" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -10571,17 +10548,16 @@
       <c r="E21" s="18" t="n">
         <v>46189.31778935185</v>
       </c>
-      <c r="F21" s="9">
-        <f>IF(OR(D21="",E21=""),"",(E21-D21)*24)</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>IF(F21="","",F21/24)</f>
-        <v/>
-      </c>
-      <c r="H21" s="19">
-        <f>IF(D21="","",TEXT(D21,"YYYY-MM"))</f>
-        <v/>
+      <c r="F21" s="9" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -10606,17 +10582,16 @@
       <c r="E22" s="18" t="n">
         <v>46189.33142361111</v>
       </c>
-      <c r="F22" s="9">
-        <f>IF(OR(D22="",E22=""),"",(E22-D22)*24)</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
-        <f>IF(F22="","",F22/24)</f>
-        <v/>
-      </c>
-      <c r="H22" s="19">
-        <f>IF(D22="","",TEXT(D22,"YYYY-MM"))</f>
-        <v/>
+      <c r="F22" s="9" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -10641,17 +10616,16 @@
       <c r="E23" s="18" t="n">
         <v>46202.489375</v>
       </c>
-      <c r="F23" s="9">
-        <f>IF(OR(D23="",E23=""),"",(E23-D23)*24)</f>
-        <v/>
-      </c>
-      <c r="G23" s="9">
-        <f>IF(F23="","",F23/24)</f>
-        <v/>
-      </c>
-      <c r="H23" s="19">
-        <f>IF(D23="","",TEXT(D23,"YYYY-MM"))</f>
-        <v/>
+      <c r="F23" s="9" t="n">
+        <v>313.8</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -10676,17 +10650,16 @@
       <c r="E24" s="18" t="n">
         <v>46190.38052083334</v>
       </c>
-      <c r="F24" s="9">
-        <f>IF(OR(D24="",E24=""),"",(E24-D24)*24)</f>
-        <v/>
-      </c>
-      <c r="G24" s="9">
-        <f>IF(F24="","",F24/24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="19">
-        <f>IF(D24="","",TEXT(D24,"YYYY-MM"))</f>
-        <v/>
+      <c r="F24" s="9" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -10711,17 +10684,16 @@
       <c r="E25" s="18" t="n">
         <v>46190.38048611111</v>
       </c>
-      <c r="F25" s="9">
-        <f>IF(OR(D25="",E25=""),"",(E25-D25)*24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="9">
-        <f>IF(F25="","",F25/24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="19">
-        <f>IF(D25="","",TEXT(D25,"YYYY-MM"))</f>
-        <v/>
+      <c r="F25" s="9" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H25" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -10746,17 +10718,16 @@
       <c r="E26" s="18" t="n">
         <v>46190.58262731481</v>
       </c>
-      <c r="F26" s="9">
-        <f>IF(OR(D26="",E26=""),"",(E26-D26)*24)</f>
-        <v/>
-      </c>
-      <c r="G26" s="9">
-        <f>IF(F26="","",F26/24)</f>
-        <v/>
-      </c>
-      <c r="H26" s="19">
-        <f>IF(D26="","",TEXT(D26,"YYYY-MM"))</f>
-        <v/>
+      <c r="F26" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -10781,17 +10752,16 @@
       <c r="E27" s="18" t="n">
         <v>46191.42747685185</v>
       </c>
-      <c r="F27" s="9">
-        <f>IF(OR(D27="",E27=""),"",(E27-D27)*24)</f>
-        <v/>
-      </c>
-      <c r="G27" s="9">
-        <f>IF(F27="","",F27/24)</f>
-        <v/>
-      </c>
-      <c r="H27" s="19">
-        <f>IF(D27="","",TEXT(D27,"YYYY-MM"))</f>
-        <v/>
+      <c r="F27" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -10816,17 +10786,16 @@
       <c r="E28" s="18" t="n">
         <v>46191.56158564815</v>
       </c>
-      <c r="F28" s="9">
-        <f>IF(OR(D28="",E28=""),"",(E28-D28)*24)</f>
-        <v/>
-      </c>
-      <c r="G28" s="9">
-        <f>IF(F28="","",F28/24)</f>
-        <v/>
-      </c>
-      <c r="H28" s="19">
-        <f>IF(D28="","",TEXT(D28,"YYYY-MM"))</f>
-        <v/>
+      <c r="F28" s="9" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -10851,17 +10820,16 @@
       <c r="E29" s="18" t="n">
         <v>46191.55452546296</v>
       </c>
-      <c r="F29" s="9">
-        <f>IF(OR(D29="",E29=""),"",(E29-D29)*24)</f>
-        <v/>
-      </c>
-      <c r="G29" s="9">
-        <f>IF(F29="","",F29/24)</f>
-        <v/>
-      </c>
-      <c r="H29" s="19">
-        <f>IF(D29="","",TEXT(D29,"YYYY-MM"))</f>
-        <v/>
+      <c r="F29" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -10886,17 +10854,16 @@
       <c r="E30" s="18" t="n">
         <v>46191.60738425926</v>
       </c>
-      <c r="F30" s="9">
-        <f>IF(OR(D30="",E30=""),"",(E30-D30)*24)</f>
-        <v/>
-      </c>
-      <c r="G30" s="9">
-        <f>IF(F30="","",F30/24)</f>
-        <v/>
-      </c>
-      <c r="H30" s="19">
-        <f>IF(D30="","",TEXT(D30,"YYYY-MM"))</f>
-        <v/>
+      <c r="F30" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -10921,17 +10888,16 @@
       <c r="E31" s="18" t="n">
         <v>46197.55138888889</v>
       </c>
-      <c r="F31" s="9">
-        <f>IF(OR(D31="",E31=""),"",(E31-D31)*24)</f>
-        <v/>
-      </c>
-      <c r="G31" s="9">
-        <f>IF(F31="","",F31/24)</f>
-        <v/>
-      </c>
-      <c r="H31" s="19">
-        <f>IF(D31="","",TEXT(D31,"YYYY-MM"))</f>
-        <v/>
+      <c r="F31" s="9" t="n">
+        <v>122.5</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -10956,17 +10922,16 @@
       <c r="E32" s="18" t="n">
         <v>46192.5315162037</v>
       </c>
-      <c r="F32" s="9">
-        <f>IF(OR(D32="",E32=""),"",(E32-D32)*24)</f>
-        <v/>
-      </c>
-      <c r="G32" s="9">
-        <f>IF(F32="","",F32/24)</f>
-        <v/>
-      </c>
-      <c r="H32" s="19">
-        <f>IF(D32="","",TEXT(D32,"YYYY-MM"))</f>
-        <v/>
+      <c r="F32" s="9" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -10991,17 +10956,16 @@
       <c r="E33" s="18" t="n">
         <v>46195.41001157407</v>
       </c>
-      <c r="F33" s="9">
-        <f>IF(OR(D33="",E33=""),"",(E33-D33)*24)</f>
-        <v/>
-      </c>
-      <c r="G33" s="9">
-        <f>IF(F33="","",F33/24)</f>
-        <v/>
-      </c>
-      <c r="H33" s="19">
-        <f>IF(D33="","",TEXT(D33,"YYYY-MM"))</f>
-        <v/>
+      <c r="F33" s="9" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -11026,17 +10990,16 @@
       <c r="E34" s="18" t="n">
         <v>46195.42172453704</v>
       </c>
-      <c r="F34" s="9">
-        <f>IF(OR(D34="",E34=""),"",(E34-D34)*24)</f>
-        <v/>
-      </c>
-      <c r="G34" s="9">
-        <f>IF(F34="","",F34/24)</f>
-        <v/>
-      </c>
-      <c r="H34" s="19">
-        <f>IF(D34="","",TEXT(D34,"YYYY-MM"))</f>
-        <v/>
+      <c r="F34" s="9" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -11061,17 +11024,16 @@
       <c r="E35" s="18" t="n">
         <v>46195.44331018518</v>
       </c>
-      <c r="F35" s="9">
-        <f>IF(OR(D35="",E35=""),"",(E35-D35)*24)</f>
-        <v/>
-      </c>
-      <c r="G35" s="9">
-        <f>IF(F35="","",F35/24)</f>
-        <v/>
-      </c>
-      <c r="H35" s="19">
-        <f>IF(D35="","",TEXT(D35,"YYYY-MM"))</f>
-        <v/>
+      <c r="F35" s="9" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="G35" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -11096,17 +11058,16 @@
       <c r="E36" s="18" t="n">
         <v>46195.42607638889</v>
       </c>
-      <c r="F36" s="9">
-        <f>IF(OR(D36="",E36=""),"",(E36-D36)*24)</f>
-        <v/>
-      </c>
-      <c r="G36" s="9">
-        <f>IF(F36="","",F36/24)</f>
-        <v/>
-      </c>
-      <c r="H36" s="19">
-        <f>IF(D36="","",TEXT(D36,"YYYY-MM"))</f>
-        <v/>
+      <c r="F36" s="9" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H36" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -11131,17 +11092,16 @@
       <c r="E37" s="18" t="n">
         <v>46195.43376157407</v>
       </c>
-      <c r="F37" s="9">
-        <f>IF(OR(D37="",E37=""),"",(E37-D37)*24)</f>
-        <v/>
-      </c>
-      <c r="G37" s="9">
-        <f>IF(F37="","",F37/24)</f>
-        <v/>
-      </c>
-      <c r="H37" s="19">
-        <f>IF(D37="","",TEXT(D37,"YYYY-MM"))</f>
-        <v/>
+      <c r="F37" s="9" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H37" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -11166,17 +11126,16 @@
       <c r="E38" s="18" t="n">
         <v>46195.4491087963</v>
       </c>
-      <c r="F38" s="9">
-        <f>IF(OR(D38="",E38=""),"",(E38-D38)*24)</f>
-        <v/>
-      </c>
-      <c r="G38" s="9">
-        <f>IF(F38="","",F38/24)</f>
-        <v/>
-      </c>
-      <c r="H38" s="19">
-        <f>IF(D38="","",TEXT(D38,"YYYY-MM"))</f>
-        <v/>
+      <c r="F38" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H38" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -11201,17 +11160,16 @@
       <c r="E39" s="18" t="n">
         <v>46196.54356481481</v>
       </c>
-      <c r="F39" s="9">
-        <f>IF(OR(D39="",E39=""),"",(E39-D39)*24)</f>
-        <v/>
-      </c>
-      <c r="G39" s="9">
-        <f>IF(F39="","",F39/24)</f>
-        <v/>
-      </c>
-      <c r="H39" s="19">
-        <f>IF(D39="","",TEXT(D39,"YYYY-MM"))</f>
-        <v/>
+      <c r="F39" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -11236,17 +11194,16 @@
       <c r="E40" s="18" t="n">
         <v>46220.59077546297</v>
       </c>
-      <c r="F40" s="9">
-        <f>IF(OR(D40="",E40=""),"",(E40-D40)*24)</f>
-        <v/>
-      </c>
-      <c r="G40" s="9">
-        <f>IF(F40="","",F40/24)</f>
-        <v/>
-      </c>
-      <c r="H40" s="19">
-        <f>IF(D40="","",TEXT(D40,"YYYY-MM"))</f>
-        <v/>
+      <c r="F40" s="9" t="n">
+        <v>576.1</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="H40" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -11271,17 +11228,16 @@
       <c r="E41" s="18" t="n">
         <v>46197.45547453704</v>
       </c>
-      <c r="F41" s="9">
-        <f>IF(OR(D41="",E41=""),"",(E41-D41)*24)</f>
-        <v/>
-      </c>
-      <c r="G41" s="9">
-        <f>IF(F41="","",F41/24)</f>
-        <v/>
-      </c>
-      <c r="H41" s="19">
-        <f>IF(D41="","",TEXT(D41,"YYYY-MM"))</f>
-        <v/>
+      <c r="F41" s="9" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H41" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -11306,17 +11262,16 @@
       <c r="E42" s="18" t="n">
         <v>46197.46196759259</v>
       </c>
-      <c r="F42" s="9">
-        <f>IF(OR(D42="",E42=""),"",(E42-D42)*24)</f>
-        <v/>
-      </c>
-      <c r="G42" s="9">
-        <f>IF(F42="","",F42/24)</f>
-        <v/>
-      </c>
-      <c r="H42" s="19">
-        <f>IF(D42="","",TEXT(D42,"YYYY-MM"))</f>
-        <v/>
+      <c r="F42" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H42" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -11341,17 +11296,16 @@
       <c r="E43" s="18" t="n">
         <v>46197.46125</v>
       </c>
-      <c r="F43" s="9">
-        <f>IF(OR(D43="",E43=""),"",(E43-D43)*24)</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>IF(F43="","",F43/24)</f>
-        <v/>
-      </c>
-      <c r="H43" s="19">
-        <f>IF(D43="","",TEXT(D43,"YYYY-MM"))</f>
-        <v/>
+      <c r="F43" s="9" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H43" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -11376,17 +11330,16 @@
       <c r="E44" s="18" t="n">
         <v>46197.47481481481</v>
       </c>
-      <c r="F44" s="9">
-        <f>IF(OR(D44="",E44=""),"",(E44-D44)*24)</f>
-        <v/>
-      </c>
-      <c r="G44" s="9">
-        <f>IF(F44="","",F44/24)</f>
-        <v/>
-      </c>
-      <c r="H44" s="19">
-        <f>IF(D44="","",TEXT(D44,"YYYY-MM"))</f>
-        <v/>
+      <c r="F44" s="9" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H44" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -11411,17 +11364,16 @@
       <c r="E45" s="18" t="n">
         <v>46198.56770833334</v>
       </c>
-      <c r="F45" s="9">
-        <f>IF(OR(D45="",E45=""),"",(E45-D45)*24)</f>
-        <v/>
-      </c>
-      <c r="G45" s="9">
-        <f>IF(F45="","",F45/24)</f>
-        <v/>
-      </c>
-      <c r="H45" s="19">
-        <f>IF(D45="","",TEXT(D45,"YYYY-MM"))</f>
-        <v/>
+      <c r="F45" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H45" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -11446,17 +11398,16 @@
       <c r="E46" s="18" t="n">
         <v>46198.59099537037</v>
       </c>
-      <c r="F46" s="9">
-        <f>IF(OR(D46="",E46=""),"",(E46-D46)*24)</f>
-        <v/>
-      </c>
-      <c r="G46" s="9">
-        <f>IF(F46="","",F46/24)</f>
-        <v/>
-      </c>
-      <c r="H46" s="19">
-        <f>IF(D46="","",TEXT(D46,"YYYY-MM"))</f>
-        <v/>
+      <c r="F46" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H46" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -11481,17 +11432,16 @@
       <c r="E47" s="18" t="n">
         <v>46198.5740625</v>
       </c>
-      <c r="F47" s="9">
-        <f>IF(OR(D47="",E47=""),"",(E47-D47)*24)</f>
-        <v/>
-      </c>
-      <c r="G47" s="9">
-        <f>IF(F47="","",F47/24)</f>
-        <v/>
-      </c>
-      <c r="H47" s="19">
-        <f>IF(D47="","",TEXT(D47,"YYYY-MM"))</f>
-        <v/>
+      <c r="F47" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -11512,17 +11462,16 @@
       <c r="E48" s="18" t="n">
         <v>46199.47065972222</v>
       </c>
-      <c r="F48" s="9">
-        <f>IF(OR(D48="",E48=""),"",(E48-D48)*24)</f>
-        <v/>
-      </c>
-      <c r="G48" s="9">
-        <f>IF(F48="","",F48/24)</f>
-        <v/>
-      </c>
-      <c r="H48" s="19">
-        <f>IF(D48="","",TEXT(D48,"YYYY-MM"))</f>
-        <v/>
+      <c r="F48" s="9" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G48" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H48" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -11547,17 +11496,16 @@
       <c r="E49" s="18" t="n">
         <v>46199.48798611111</v>
       </c>
-      <c r="F49" s="9">
-        <f>IF(OR(D49="",E49=""),"",(E49-D49)*24)</f>
-        <v/>
-      </c>
-      <c r="G49" s="9">
-        <f>IF(F49="","",F49/24)</f>
-        <v/>
-      </c>
-      <c r="H49" s="19">
-        <f>IF(D49="","",TEXT(D49,"YYYY-MM"))</f>
-        <v/>
+      <c r="F49" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G49" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -11582,17 +11530,16 @@
       <c r="E50" s="18" t="n">
         <v>46202.54658564815</v>
       </c>
-      <c r="F50" s="9">
-        <f>IF(OR(D50="",E50=""),"",(E50-D50)*24)</f>
-        <v/>
-      </c>
-      <c r="G50" s="9">
-        <f>IF(F50="","",F50/24)</f>
-        <v/>
-      </c>
-      <c r="H50" s="19">
-        <f>IF(D50="","",TEXT(D50,"YYYY-MM"))</f>
-        <v/>
+      <c r="F50" s="9" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H50" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -11617,17 +11564,16 @@
       <c r="E51" s="18" t="n">
         <v>46202.5175</v>
       </c>
-      <c r="F51" s="9">
-        <f>IF(OR(D51="",E51=""),"",(E51-D51)*24)</f>
-        <v/>
-      </c>
-      <c r="G51" s="9">
-        <f>IF(F51="","",F51/24)</f>
-        <v/>
-      </c>
-      <c r="H51" s="19">
-        <f>IF(D51="","",TEXT(D51,"YYYY-MM"))</f>
-        <v/>
+      <c r="F51" s="9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G51" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -11652,17 +11598,16 @@
       <c r="E52" s="18" t="n">
         <v>46202.62076388889</v>
       </c>
-      <c r="F52" s="9">
-        <f>IF(OR(D52="",E52=""),"",(E52-D52)*24)</f>
-        <v/>
-      </c>
-      <c r="G52" s="9">
-        <f>IF(F52="","",F52/24)</f>
-        <v/>
-      </c>
-      <c r="H52" s="19">
-        <f>IF(D52="","",TEXT(D52,"YYYY-MM"))</f>
-        <v/>
+      <c r="F52" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H52" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -11687,17 +11632,16 @@
       <c r="E53" s="18" t="n">
         <v>46202.93710648148</v>
       </c>
-      <c r="F53" s="9">
-        <f>IF(OR(D53="",E53=""),"",(E53-D53)*24)</f>
-        <v/>
-      </c>
-      <c r="G53" s="9">
-        <f>IF(F53="","",F53/24)</f>
-        <v/>
-      </c>
-      <c r="H53" s="19">
-        <f>IF(D53="","",TEXT(D53,"YYYY-MM"))</f>
-        <v/>
+      <c r="F53" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="G53" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -11722,17 +11666,16 @@
       <c r="E54" s="18" t="n">
         <v>46202.91690972223</v>
       </c>
-      <c r="F54" s="9">
-        <f>IF(OR(D54="",E54=""),"",(E54-D54)*24)</f>
-        <v/>
-      </c>
-      <c r="G54" s="9">
-        <f>IF(F54="","",F54/24)</f>
-        <v/>
-      </c>
-      <c r="H54" s="19">
-        <f>IF(D54="","",TEXT(D54,"YYYY-MM"))</f>
-        <v/>
+      <c r="F54" s="9" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H54" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -11757,17 +11700,16 @@
       <c r="E55" s="18" t="n">
         <v>46202.93311342593</v>
       </c>
-      <c r="F55" s="9">
-        <f>IF(OR(D55="",E55=""),"",(E55-D55)*24)</f>
-        <v/>
-      </c>
-      <c r="G55" s="9">
-        <f>IF(F55="","",F55/24)</f>
-        <v/>
-      </c>
-      <c r="H55" s="19">
-        <f>IF(D55="","",TEXT(D55,"YYYY-MM"))</f>
-        <v/>
+      <c r="F55" s="9" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H55" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -11792,17 +11734,16 @@
       <c r="E56" s="18" t="n">
         <v>46202.92932870371</v>
       </c>
-      <c r="F56" s="9">
-        <f>IF(OR(D56="",E56=""),"",(E56-D56)*24)</f>
-        <v/>
-      </c>
-      <c r="G56" s="9">
-        <f>IF(F56="","",F56/24)</f>
-        <v/>
-      </c>
-      <c r="H56" s="19">
-        <f>IF(D56="","",TEXT(D56,"YYYY-MM"))</f>
-        <v/>
+      <c r="F56" s="9" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H56" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -11827,17 +11768,16 @@
       <c r="E57" s="18" t="n">
         <v>46210.34105324074</v>
       </c>
-      <c r="F57" s="9">
-        <f>IF(OR(D57="",E57=""),"",(E57-D57)*24)</f>
-        <v/>
-      </c>
-      <c r="G57" s="9">
-        <f>IF(F57="","",F57/24)</f>
-        <v/>
-      </c>
-      <c r="H57" s="19">
-        <f>IF(D57="","",TEXT(D57,"YYYY-MM"))</f>
-        <v/>
+      <c r="F57" s="9" t="n">
+        <v>181.1</v>
+      </c>
+      <c r="G57" s="9" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -11862,17 +11802,16 @@
       <c r="E58" s="18" t="n">
         <v>46202.89962962963</v>
       </c>
-      <c r="F58" s="9">
-        <f>IF(OR(D58="",E58=""),"",(E58-D58)*24)</f>
-        <v/>
-      </c>
-      <c r="G58" s="9">
-        <f>IF(F58="","",F58/24)</f>
-        <v/>
-      </c>
-      <c r="H58" s="19">
-        <f>IF(D58="","",TEXT(D58,"YYYY-MM"))</f>
-        <v/>
+      <c r="F58" s="9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G58" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -11897,17 +11836,16 @@
       <c r="E59" s="18" t="n">
         <v>46218.47298611111</v>
       </c>
-      <c r="F59" s="9">
-        <f>IF(OR(D59="",E59=""),"",(E59-D59)*24)</f>
-        <v/>
-      </c>
-      <c r="G59" s="9">
-        <f>IF(F59="","",F59/24)</f>
-        <v/>
-      </c>
-      <c r="H59" s="19">
-        <f>IF(D59="","",TEXT(D59,"YYYY-MM"))</f>
-        <v/>
+      <c r="F59" s="9" t="n">
+        <v>360.3</v>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -11932,17 +11870,16 @@
       <c r="E60" s="18" t="n">
         <v>46204.50627314814</v>
       </c>
-      <c r="F60" s="9">
-        <f>IF(OR(D60="",E60=""),"",(E60-D60)*24)</f>
-        <v/>
-      </c>
-      <c r="G60" s="9">
-        <f>IF(F60="","",F60/24)</f>
-        <v/>
-      </c>
-      <c r="H60" s="19">
-        <f>IF(D60="","",TEXT(D60,"YYYY-MM"))</f>
-        <v/>
+      <c r="F60" s="9" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -11967,17 +11904,16 @@
       <c r="E61" s="18" t="n">
         <v>46204.42306712963</v>
       </c>
-      <c r="F61" s="9">
-        <f>IF(OR(D61="",E61=""),"",(E61-D61)*24)</f>
-        <v/>
-      </c>
-      <c r="G61" s="9">
-        <f>IF(F61="","",F61/24)</f>
-        <v/>
-      </c>
-      <c r="H61" s="19">
-        <f>IF(D61="","",TEXT(D61,"YYYY-MM"))</f>
-        <v/>
+      <c r="F61" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G61" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -12002,17 +11938,16 @@
       <c r="E62" s="18" t="n">
         <v>46209.48625</v>
       </c>
-      <c r="F62" s="9">
-        <f>IF(OR(D62="",E62=""),"",(E62-D62)*24)</f>
-        <v/>
-      </c>
-      <c r="G62" s="9">
-        <f>IF(F62="","",F62/24)</f>
-        <v/>
-      </c>
-      <c r="H62" s="19">
-        <f>IF(D62="","",TEXT(D62,"YYYY-MM"))</f>
-        <v/>
+      <c r="F62" s="9" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -12037,17 +11972,16 @@
       <c r="E63" s="18" t="n">
         <v>46204.61782407408</v>
       </c>
-      <c r="F63" s="9">
-        <f>IF(OR(D63="",E63=""),"",(E63-D63)*24)</f>
-        <v/>
-      </c>
-      <c r="G63" s="9">
-        <f>IF(F63="","",F63/24)</f>
-        <v/>
-      </c>
-      <c r="H63" s="19">
-        <f>IF(D63="","",TEXT(D63,"YYYY-MM"))</f>
-        <v/>
+      <c r="F63" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G63" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -12072,17 +12006,16 @@
       <c r="E64" s="18" t="n">
         <v>46205.411875</v>
       </c>
-      <c r="F64" s="9">
-        <f>IF(OR(D64="",E64=""),"",(E64-D64)*24)</f>
-        <v/>
-      </c>
-      <c r="G64" s="9">
-        <f>IF(F64="","",F64/24)</f>
-        <v/>
-      </c>
-      <c r="H64" s="19">
-        <f>IF(D64="","",TEXT(D64,"YYYY-MM"))</f>
-        <v/>
+      <c r="F64" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H64" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -12107,17 +12040,16 @@
       <c r="E65" s="18" t="n">
         <v>46206.39912037037</v>
       </c>
-      <c r="F65" s="9">
-        <f>IF(OR(D65="",E65=""),"",(E65-D65)*24)</f>
-        <v/>
-      </c>
-      <c r="G65" s="9">
-        <f>IF(F65="","",F65/24)</f>
-        <v/>
-      </c>
-      <c r="H65" s="19">
-        <f>IF(D65="","",TEXT(D65,"YYYY-MM"))</f>
-        <v/>
+      <c r="F65" s="9" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H65" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -12142,17 +12074,16 @@
       <c r="E66" s="18" t="n">
         <v>46206.44606481482</v>
       </c>
-      <c r="F66" s="9">
-        <f>IF(OR(D66="",E66=""),"",(E66-D66)*24)</f>
-        <v/>
-      </c>
-      <c r="G66" s="9">
-        <f>IF(F66="","",F66/24)</f>
-        <v/>
-      </c>
-      <c r="H66" s="19">
-        <f>IF(D66="","",TEXT(D66,"YYYY-MM"))</f>
-        <v/>
+      <c r="F66" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H66" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -12177,17 +12108,16 @@
       <c r="E67" s="18" t="n">
         <v>46206.44741898148</v>
       </c>
-      <c r="F67" s="9">
-        <f>IF(OR(D67="",E67=""),"",(E67-D67)*24)</f>
-        <v/>
-      </c>
-      <c r="G67" s="9">
-        <f>IF(F67="","",F67/24)</f>
-        <v/>
-      </c>
-      <c r="H67" s="19">
-        <f>IF(D67="","",TEXT(D67,"YYYY-MM"))</f>
-        <v/>
+      <c r="F67" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G67" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -12212,17 +12142,16 @@
       <c r="E68" s="18" t="n">
         <v>46206.45150462963</v>
       </c>
-      <c r="F68" s="9">
-        <f>IF(OR(D68="",E68=""),"",(E68-D68)*24)</f>
-        <v/>
-      </c>
-      <c r="G68" s="9">
-        <f>IF(F68="","",F68/24)</f>
-        <v/>
-      </c>
-      <c r="H68" s="19">
-        <f>IF(D68="","",TEXT(D68,"YYYY-MM"))</f>
-        <v/>
+      <c r="F68" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -12247,17 +12176,16 @@
       <c r="E69" s="18" t="n">
         <v>46206.51376157408</v>
       </c>
-      <c r="F69" s="9">
-        <f>IF(OR(D69="",E69=""),"",(E69-D69)*24)</f>
-        <v/>
-      </c>
-      <c r="G69" s="9">
-        <f>IF(F69="","",F69/24)</f>
-        <v/>
-      </c>
-      <c r="H69" s="19">
-        <f>IF(D69="","",TEXT(D69,"YYYY-MM"))</f>
-        <v/>
+      <c r="F69" s="9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G69" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H69" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -12282,17 +12210,16 @@
       <c r="E70" s="18" t="n">
         <v>46245.38761574074</v>
       </c>
-      <c r="F70" s="9">
-        <f>IF(OR(D70="",E70=""),"",(E70-D70)*24)</f>
-        <v/>
-      </c>
-      <c r="G70" s="9">
-        <f>IF(F70="","",F70/24)</f>
-        <v/>
-      </c>
-      <c r="H70" s="19">
-        <f>IF(D70="","",TEXT(D70,"YYYY-MM"))</f>
-        <v/>
+      <c r="F70" s="9" t="n">
+        <v>934.8</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="H70" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -12317,17 +12244,16 @@
       <c r="E71" s="18" t="n">
         <v>46209.46458333333</v>
       </c>
-      <c r="F71" s="9">
-        <f>IF(OR(D71="",E71=""),"",(E71-D71)*24)</f>
-        <v/>
-      </c>
-      <c r="G71" s="9">
-        <f>IF(F71="","",F71/24)</f>
-        <v/>
-      </c>
-      <c r="H71" s="19">
-        <f>IF(D71="","",TEXT(D71,"YYYY-MM"))</f>
-        <v/>
+      <c r="F71" s="9" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="G71" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H71" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -12352,17 +12278,16 @@
       <c r="E72" s="18" t="n">
         <v>46209.46138888889</v>
       </c>
-      <c r="F72" s="9">
-        <f>IF(OR(D72="",E72=""),"",(E72-D72)*24)</f>
-        <v/>
-      </c>
-      <c r="G72" s="9">
-        <f>IF(F72="","",F72/24)</f>
-        <v/>
-      </c>
-      <c r="H72" s="19">
-        <f>IF(D72="","",TEXT(D72,"YYYY-MM"))</f>
-        <v/>
+      <c r="F72" s="9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H72" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -12387,17 +12312,16 @@
       <c r="E73" s="18" t="n">
         <v>46231.49832175926</v>
       </c>
-      <c r="F73" s="9">
-        <f>IF(OR(D73="",E73=""),"",(E73-D73)*24)</f>
-        <v/>
-      </c>
-      <c r="G73" s="9">
-        <f>IF(F73="","",F73/24)</f>
-        <v/>
-      </c>
-      <c r="H73" s="19">
-        <f>IF(D73="","",TEXT(D73,"YYYY-MM"))</f>
-        <v/>
+      <c r="F73" s="9" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="G73" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H73" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -12422,17 +12346,16 @@
       <c r="E74" s="18" t="n">
         <v>46231.49868055555</v>
       </c>
-      <c r="F74" s="9">
-        <f>IF(OR(D74="",E74=""),"",(E74-D74)*24)</f>
-        <v/>
-      </c>
-      <c r="G74" s="9">
-        <f>IF(F74="","",F74/24)</f>
-        <v/>
-      </c>
-      <c r="H74" s="19">
-        <f>IF(D74="","",TEXT(D74,"YYYY-MM"))</f>
-        <v/>
+      <c r="F74" s="9" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="H74" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -12457,17 +12380,16 @@
       <c r="E75" s="18" t="n">
         <v>46211.60092592592</v>
       </c>
-      <c r="F75" s="9">
-        <f>IF(OR(D75="",E75=""),"",(E75-D75)*24)</f>
-        <v/>
-      </c>
-      <c r="G75" s="9">
-        <f>IF(F75="","",F75/24)</f>
-        <v/>
-      </c>
-      <c r="H75" s="19">
-        <f>IF(D75="","",TEXT(D75,"YYYY-MM"))</f>
-        <v/>
+      <c r="F75" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G75" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -12492,17 +12414,16 @@
       <c r="E76" s="18" t="n">
         <v>46211.61304398148</v>
       </c>
-      <c r="F76" s="9">
-        <f>IF(OR(D76="",E76=""),"",(E76-D76)*24)</f>
-        <v/>
-      </c>
-      <c r="G76" s="9">
-        <f>IF(F76="","",F76/24)</f>
-        <v/>
-      </c>
-      <c r="H76" s="19">
-        <f>IF(D76="","",TEXT(D76,"YYYY-MM"))</f>
-        <v/>
+      <c r="F76" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -12527,17 +12448,16 @@
       <c r="E77" s="18" t="n">
         <v>46211.61459490741</v>
       </c>
-      <c r="F77" s="9">
-        <f>IF(OR(D77="",E77=""),"",(E77-D77)*24)</f>
-        <v/>
-      </c>
-      <c r="G77" s="9">
-        <f>IF(F77="","",F77/24)</f>
-        <v/>
-      </c>
-      <c r="H77" s="19">
-        <f>IF(D77="","",TEXT(D77,"YYYY-MM"))</f>
-        <v/>
+      <c r="F77" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G77" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -12562,17 +12482,16 @@
       <c r="E78" s="18" t="n">
         <v>46212.48398148148</v>
       </c>
-      <c r="F78" s="9">
-        <f>IF(OR(D78="",E78=""),"",(E78-D78)*24)</f>
-        <v/>
-      </c>
-      <c r="G78" s="9">
-        <f>IF(F78="","",F78/24)</f>
-        <v/>
-      </c>
-      <c r="H78" s="19">
-        <f>IF(D78="","",TEXT(D78,"YYYY-MM"))</f>
-        <v/>
+      <c r="F78" s="9" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H78" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -12597,17 +12516,16 @@
       <c r="E79" s="18" t="n">
         <v>46213.49804398148</v>
       </c>
-      <c r="F79" s="9">
-        <f>IF(OR(D79="",E79=""),"",(E79-D79)*24)</f>
-        <v/>
-      </c>
-      <c r="G79" s="9">
-        <f>IF(F79="","",F79/24)</f>
-        <v/>
-      </c>
-      <c r="H79" s="19">
-        <f>IF(D79="","",TEXT(D79,"YYYY-MM"))</f>
-        <v/>
+      <c r="F79" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H79" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -12628,17 +12546,16 @@
       <c r="E80" s="18" t="n">
         <v>46216.50620370371</v>
       </c>
-      <c r="F80" s="9">
-        <f>IF(OR(D80="",E80=""),"",(E80-D80)*24)</f>
-        <v/>
-      </c>
-      <c r="G80" s="9">
-        <f>IF(F80="","",F80/24)</f>
-        <v/>
-      </c>
-      <c r="H80" s="19">
-        <f>IF(D80="","",TEXT(D80,"YYYY-MM"))</f>
-        <v/>
+      <c r="F80" s="9" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H80" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -12663,17 +12580,16 @@
       <c r="E81" s="18" t="n">
         <v>46216.50920138889</v>
       </c>
-      <c r="F81" s="9">
-        <f>IF(OR(D81="",E81=""),"",(E81-D81)*24)</f>
-        <v/>
-      </c>
-      <c r="G81" s="9">
-        <f>IF(F81="","",F81/24)</f>
-        <v/>
-      </c>
-      <c r="H81" s="19">
-        <f>IF(D81="","",TEXT(D81,"YYYY-MM"))</f>
-        <v/>
+      <c r="F81" s="9" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G81" s="9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H81" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -12698,17 +12614,16 @@
       <c r="E82" s="18" t="n">
         <v>46218.46796296296</v>
       </c>
-      <c r="F82" s="9">
-        <f>IF(OR(D82="",E82=""),"",(E82-D82)*24)</f>
-        <v/>
-      </c>
-      <c r="G82" s="9">
-        <f>IF(F82="","",F82/24)</f>
-        <v/>
-      </c>
-      <c r="H82" s="19">
-        <f>IF(D82="","",TEXT(D82,"YYYY-MM"))</f>
-        <v/>
+      <c r="F82" s="9" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H82" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -12733,17 +12648,16 @@
       <c r="E83" s="18" t="n">
         <v>46216.51510416667</v>
       </c>
-      <c r="F83" s="9">
-        <f>IF(OR(D83="",E83=""),"",(E83-D83)*24)</f>
-        <v/>
-      </c>
-      <c r="G83" s="9">
-        <f>IF(F83="","",F83/24)</f>
-        <v/>
-      </c>
-      <c r="H83" s="19">
-        <f>IF(D83="","",TEXT(D83,"YYYY-MM"))</f>
-        <v/>
+      <c r="F83" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H83" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -12768,17 +12682,16 @@
       <c r="E84" s="18" t="n">
         <v>46216.60158564815</v>
       </c>
-      <c r="F84" s="9">
-        <f>IF(OR(D84="",E84=""),"",(E84-D84)*24)</f>
-        <v/>
-      </c>
-      <c r="G84" s="9">
-        <f>IF(F84="","",F84/24)</f>
-        <v/>
-      </c>
-      <c r="H84" s="19">
-        <f>IF(D84="","",TEXT(D84,"YYYY-MM"))</f>
-        <v/>
+      <c r="F84" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -12803,17 +12716,16 @@
       <c r="E85" s="18" t="n">
         <v>46218.46759259259</v>
       </c>
-      <c r="F85" s="9">
-        <f>IF(OR(D85="",E85=""),"",(E85-D85)*24)</f>
-        <v/>
-      </c>
-      <c r="G85" s="9">
-        <f>IF(F85="","",F85/24)</f>
-        <v/>
-      </c>
-      <c r="H85" s="19">
-        <f>IF(D85="","",TEXT(D85,"YYYY-MM"))</f>
-        <v/>
+      <c r="F85" s="9" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H85" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -12838,17 +12750,16 @@
       <c r="E86" s="18" t="n">
         <v>46218.55229166667</v>
       </c>
-      <c r="F86" s="9">
-        <f>IF(OR(D86="",E86=""),"",(E86-D86)*24)</f>
-        <v/>
-      </c>
-      <c r="G86" s="9">
-        <f>IF(F86="","",F86/24)</f>
-        <v/>
-      </c>
-      <c r="H86" s="19">
-        <f>IF(D86="","",TEXT(D86,"YYYY-MM"))</f>
-        <v/>
+      <c r="F86" s="9" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H86" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -12873,17 +12784,16 @@
       <c r="E87" s="18" t="n">
         <v>46245.38123842593</v>
       </c>
-      <c r="F87" s="9">
-        <f>IF(OR(D87="",E87=""),"",(E87-D87)*24)</f>
-        <v/>
-      </c>
-      <c r="G87" s="9">
-        <f>IF(F87="","",F87/24)</f>
-        <v/>
-      </c>
-      <c r="H87" s="19">
-        <f>IF(D87="","",TEXT(D87,"YYYY-MM"))</f>
-        <v/>
+      <c r="F87" s="9" t="n">
+        <v>670.4</v>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="H87" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -12908,17 +12818,16 @@
       <c r="E88" s="18" t="n">
         <v>46219.59121527777</v>
       </c>
-      <c r="F88" s="9">
-        <f>IF(OR(D88="",E88=""),"",(E88-D88)*24)</f>
-        <v/>
-      </c>
-      <c r="G88" s="9">
-        <f>IF(F88="","",F88/24)</f>
-        <v/>
-      </c>
-      <c r="H88" s="19">
-        <f>IF(D88="","",TEXT(D88,"YYYY-MM"))</f>
-        <v/>
+      <c r="F88" s="9" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H88" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -12943,17 +12852,16 @@
       <c r="E89" s="18" t="n">
         <v>46223.59344907408</v>
       </c>
-      <c r="F89" s="9">
-        <f>IF(OR(D89="",E89=""),"",(E89-D89)*24)</f>
-        <v/>
-      </c>
-      <c r="G89" s="9">
-        <f>IF(F89="","",F89/24)</f>
-        <v/>
-      </c>
-      <c r="H89" s="19">
-        <f>IF(D89="","",TEXT(D89,"YYYY-MM"))</f>
-        <v/>
+      <c r="F89" s="9" t="n">
+        <v>96.3</v>
+      </c>
+      <c r="G89" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H89" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -12978,17 +12886,16 @@
       <c r="E90" s="18" t="n">
         <v>46223.59318287037</v>
       </c>
-      <c r="F90" s="9">
-        <f>IF(OR(D90="",E90=""),"",(E90-D90)*24)</f>
-        <v/>
-      </c>
-      <c r="G90" s="9">
-        <f>IF(F90="","",F90/24)</f>
-        <v/>
-      </c>
-      <c r="H90" s="19">
-        <f>IF(D90="","",TEXT(D90,"YYYY-MM"))</f>
-        <v/>
+      <c r="F90" s="9" t="n">
+        <v>71.90000000000001</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H90" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -13013,17 +12920,16 @@
       <c r="E91" s="18" t="n">
         <v>46223.59586805556</v>
       </c>
-      <c r="F91" s="9">
-        <f>IF(OR(D91="",E91=""),"",(E91-D91)*24)</f>
-        <v/>
-      </c>
-      <c r="G91" s="9">
-        <f>IF(F91="","",F91/24)</f>
-        <v/>
-      </c>
-      <c r="H91" s="19">
-        <f>IF(D91="","",TEXT(D91,"YYYY-MM"))</f>
-        <v/>
+      <c r="F91" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -13048,17 +12954,16 @@
       <c r="E92" s="18" t="n">
         <v>46224.44824074074</v>
       </c>
-      <c r="F92" s="9">
-        <f>IF(OR(D92="",E92=""),"",(E92-D92)*24)</f>
-        <v/>
-      </c>
-      <c r="G92" s="9">
-        <f>IF(F92="","",F92/24)</f>
-        <v/>
-      </c>
-      <c r="H92" s="19">
-        <f>IF(D92="","",TEXT(D92,"YYYY-MM"))</f>
-        <v/>
+      <c r="F92" s="9" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H92" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -13083,17 +12988,16 @@
       <c r="E93" s="18" t="n">
         <v>46224.53614583334</v>
       </c>
-      <c r="F93" s="9">
-        <f>IF(OR(D93="",E93=""),"",(E93-D93)*24)</f>
-        <v/>
-      </c>
-      <c r="G93" s="9">
-        <f>IF(F93="","",F93/24)</f>
-        <v/>
-      </c>
-      <c r="H93" s="19">
-        <f>IF(D93="","",TEXT(D93,"YYYY-MM"))</f>
-        <v/>
+      <c r="F93" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H93" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -13118,17 +13022,16 @@
       <c r="E94" s="18" t="n">
         <v>46224.46887731482</v>
       </c>
-      <c r="F94" s="9">
-        <f>IF(OR(D94="",E94=""),"",(E94-D94)*24)</f>
-        <v/>
-      </c>
-      <c r="G94" s="9">
-        <f>IF(F94="","",F94/24)</f>
-        <v/>
-      </c>
-      <c r="H94" s="19">
-        <f>IF(D94="","",TEXT(D94,"YYYY-MM"))</f>
-        <v/>
+      <c r="F94" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -13153,17 +13056,16 @@
       <c r="E95" s="18" t="n">
         <v>46226.39471064815</v>
       </c>
-      <c r="F95" s="9">
-        <f>IF(OR(D95="",E95=""),"",(E95-D95)*24)</f>
-        <v/>
-      </c>
-      <c r="G95" s="9">
-        <f>IF(F95="","",F95/24)</f>
-        <v/>
-      </c>
-      <c r="H95" s="19">
-        <f>IF(D95="","",TEXT(D95,"YYYY-MM"))</f>
-        <v/>
+      <c r="F95" s="9" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H95" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -13188,17 +13090,16 @@
       <c r="E96" s="18" t="n">
         <v>46225.56233796296</v>
       </c>
-      <c r="F96" s="9">
-        <f>IF(OR(D96="",E96=""),"",(E96-D96)*24)</f>
-        <v/>
-      </c>
-      <c r="G96" s="9">
-        <f>IF(F96="","",F96/24)</f>
-        <v/>
-      </c>
-      <c r="H96" s="19">
-        <f>IF(D96="","",TEXT(D96,"YYYY-MM"))</f>
-        <v/>
+      <c r="F96" s="9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H96" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -13223,17 +13124,16 @@
       <c r="E97" s="18" t="n">
         <v>46226.40005787037</v>
       </c>
-      <c r="F97" s="9">
-        <f>IF(OR(D97="",E97=""),"",(E97-D97)*24)</f>
-        <v/>
-      </c>
-      <c r="G97" s="9">
-        <f>IF(F97="","",F97/24)</f>
-        <v/>
-      </c>
-      <c r="H97" s="19">
-        <f>IF(D97="","",TEXT(D97,"YYYY-MM"))</f>
-        <v/>
+      <c r="F97" s="9" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H97" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -13258,17 +13158,16 @@
       <c r="E98" s="18" t="n">
         <v>46227.34571759259</v>
       </c>
-      <c r="F98" s="9">
-        <f>IF(OR(D98="",E98=""),"",(E98-D98)*24)</f>
-        <v/>
-      </c>
-      <c r="G98" s="9">
-        <f>IF(F98="","",F98/24)</f>
-        <v/>
-      </c>
-      <c r="H98" s="19">
-        <f>IF(D98="","",TEXT(D98,"YYYY-MM"))</f>
-        <v/>
+      <c r="F98" s="9" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H98" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -13293,17 +13192,16 @@
       <c r="E99" s="18" t="n">
         <v>46245.38356481482</v>
       </c>
-      <c r="F99" s="9">
-        <f>IF(OR(D99="",E99=""),"",(E99-D99)*24)</f>
-        <v/>
-      </c>
-      <c r="G99" s="9">
-        <f>IF(F99="","",F99/24)</f>
-        <v/>
-      </c>
-      <c r="H99" s="19">
-        <f>IF(D99="","",TEXT(D99,"YYYY-MM"))</f>
-        <v/>
+      <c r="F99" s="9" t="n">
+        <v>454</v>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H99" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -13328,17 +13226,16 @@
       <c r="E100" s="18" t="n">
         <v>46227.42974537037</v>
       </c>
-      <c r="F100" s="9">
-        <f>IF(OR(D100="",E100=""),"",(E100-D100)*24)</f>
-        <v/>
-      </c>
-      <c r="G100" s="9">
-        <f>IF(F100="","",F100/24)</f>
-        <v/>
-      </c>
-      <c r="H100" s="19">
-        <f>IF(D100="","",TEXT(D100,"YYYY-MM"))</f>
-        <v/>
+      <c r="F100" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H100" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -13363,17 +13260,16 @@
       <c r="E101" s="18" t="n">
         <v>46227.57420138889</v>
       </c>
-      <c r="F101" s="9">
-        <f>IF(OR(D101="",E101=""),"",(E101-D101)*24)</f>
-        <v/>
-      </c>
-      <c r="G101" s="9">
-        <f>IF(F101="","",F101/24)</f>
-        <v/>
-      </c>
-      <c r="H101" s="19">
-        <f>IF(D101="","",TEXT(D101,"YYYY-MM"))</f>
-        <v/>
+      <c r="F101" s="9" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H101" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -13398,17 +13294,16 @@
       <c r="E102" s="18" t="n">
         <v>46245.38488425926</v>
       </c>
-      <c r="F102" s="9">
-        <f>IF(OR(D102="",E102=""),"",(E102-D102)*24)</f>
-        <v/>
-      </c>
-      <c r="G102" s="9">
-        <f>IF(F102="","",F102/24)</f>
-        <v/>
-      </c>
-      <c r="H102" s="19">
-        <f>IF(D102="","",TEXT(D102,"YYYY-MM"))</f>
-        <v/>
+      <c r="F102" s="9" t="n">
+        <v>427.4</v>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="H102" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -13433,17 +13328,16 @@
       <c r="E103" s="18" t="n">
         <v>46230.459375</v>
       </c>
-      <c r="F103" s="9">
-        <f>IF(OR(D103="",E103=""),"",(E103-D103)*24)</f>
-        <v/>
-      </c>
-      <c r="G103" s="9">
-        <f>IF(F103="","",F103/24)</f>
-        <v/>
-      </c>
-      <c r="H103" s="19">
-        <f>IF(D103="","",TEXT(D103,"YYYY-MM"))</f>
-        <v/>
+      <c r="F103" s="9" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="G103" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H103" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -13458,17 +13352,12 @@
         <v>46230.40052083333</v>
       </c>
       <c r="E104" s="18" t="n"/>
-      <c r="F104" s="9">
-        <f>IF(OR(D104="",E104=""),"",(E104-D104)*24)</f>
-        <v/>
-      </c>
-      <c r="G104" s="9">
-        <f>IF(F104="","",F104/24)</f>
-        <v/>
-      </c>
-      <c r="H104" s="19">
-        <f>IF(D104="","",TEXT(D104,"YYYY-MM"))</f>
-        <v/>
+      <c r="F104" s="9" t="n"/>
+      <c r="G104" s="9" t="n"/>
+      <c r="H104" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -13493,17 +13382,16 @@
       <c r="E105" s="18" t="n">
         <v>46230.49866898148</v>
       </c>
-      <c r="F105" s="9">
-        <f>IF(OR(D105="",E105=""),"",(E105-D105)*24)</f>
-        <v/>
-      </c>
-      <c r="G105" s="9">
-        <f>IF(F105="","",F105/24)</f>
-        <v/>
-      </c>
-      <c r="H105" s="19">
-        <f>IF(D105="","",TEXT(D105,"YYYY-MM"))</f>
-        <v/>
+      <c r="F105" s="9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H105" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -13528,17 +13416,16 @@
       <c r="E106" s="18" t="n">
         <v>46230.47216435185</v>
       </c>
-      <c r="F106" s="9">
-        <f>IF(OR(D106="",E106=""),"",(E106-D106)*24)</f>
-        <v/>
-      </c>
-      <c r="G106" s="9">
-        <f>IF(F106="","",F106/24)</f>
-        <v/>
-      </c>
-      <c r="H106" s="19">
-        <f>IF(D106="","",TEXT(D106,"YYYY-MM"))</f>
-        <v/>
+      <c r="F106" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="107">
@@ -13563,17 +13450,16 @@
       <c r="E107" s="18" t="n">
         <v>46231.34666666666</v>
       </c>
-      <c r="F107" s="9">
-        <f>IF(OR(D107="",E107=""),"",(E107-D107)*24)</f>
-        <v/>
-      </c>
-      <c r="G107" s="9">
-        <f>IF(F107="","",F107/24)</f>
-        <v/>
-      </c>
-      <c r="H107" s="19">
-        <f>IF(D107="","",TEXT(D107,"YYYY-MM"))</f>
-        <v/>
+      <c r="F107" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="108">
@@ -13598,17 +13484,16 @@
       <c r="E108" s="18" t="n">
         <v>46232.57114583333</v>
       </c>
-      <c r="F108" s="9">
-        <f>IF(OR(D108="",E108=""),"",(E108-D108)*24)</f>
-        <v/>
-      </c>
-      <c r="G108" s="9">
-        <f>IF(F108="","",F108/24)</f>
-        <v/>
-      </c>
-      <c r="H108" s="19">
-        <f>IF(D108="","",TEXT(D108,"YYYY-MM"))</f>
-        <v/>
+      <c r="F108" s="9" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="109">
@@ -13633,17 +13518,16 @@
       <c r="E109" s="18" t="n">
         <v>46232.58498842592</v>
       </c>
-      <c r="F109" s="9">
-        <f>IF(OR(D109="",E109=""),"",(E109-D109)*24)</f>
-        <v/>
-      </c>
-      <c r="G109" s="9">
-        <f>IF(F109="","",F109/24)</f>
-        <v/>
-      </c>
-      <c r="H109" s="19">
-        <f>IF(D109="","",TEXT(D109,"YYYY-MM"))</f>
-        <v/>
+      <c r="F109" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G109" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="110">
@@ -13668,17 +13552,16 @@
       <c r="E110" s="18" t="n">
         <v>46233.34712962963</v>
       </c>
-      <c r="F110" s="9">
-        <f>IF(OR(D110="",E110=""),"",(E110-D110)*24)</f>
-        <v/>
-      </c>
-      <c r="G110" s="9">
-        <f>IF(F110="","",F110/24)</f>
-        <v/>
-      </c>
-      <c r="H110" s="19">
-        <f>IF(D110="","",TEXT(D110,"YYYY-MM"))</f>
-        <v/>
+      <c r="F110" s="9" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G110" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H110" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="111">
@@ -13703,17 +13586,16 @@
       <c r="E111" s="18" t="n">
         <v>46233.3384375</v>
       </c>
-      <c r="F111" s="9">
-        <f>IF(OR(D111="",E111=""),"",(E111-D111)*24)</f>
-        <v/>
-      </c>
-      <c r="G111" s="9">
-        <f>IF(F111="","",F111/24)</f>
-        <v/>
-      </c>
-      <c r="H111" s="19">
-        <f>IF(D111="","",TEXT(D111,"YYYY-MM"))</f>
-        <v/>
+      <c r="F111" s="9" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G111" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H111" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="112">
@@ -13738,17 +13620,16 @@
       <c r="E112" s="18" t="n">
         <v>46233.56813657407</v>
       </c>
-      <c r="F112" s="9">
-        <f>IF(OR(D112="",E112=""),"",(E112-D112)*24)</f>
-        <v/>
-      </c>
-      <c r="G112" s="9">
-        <f>IF(F112="","",F112/24)</f>
-        <v/>
-      </c>
-      <c r="H112" s="19">
-        <f>IF(D112="","",TEXT(D112,"YYYY-MM"))</f>
-        <v/>
+      <c r="F112" s="9" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G112" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H112" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="113">
@@ -13769,17 +13650,16 @@
       <c r="E113" s="18" t="n">
         <v>46234.42414351852</v>
       </c>
-      <c r="F113" s="9">
-        <f>IF(OR(D113="",E113=""),"",(E113-D113)*24)</f>
-        <v/>
-      </c>
-      <c r="G113" s="9">
-        <f>IF(F113="","",F113/24)</f>
-        <v/>
-      </c>
-      <c r="H113" s="19">
-        <f>IF(D113="","",TEXT(D113,"YYYY-MM"))</f>
-        <v/>
+      <c r="F113" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G113" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H113" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="114">
@@ -13800,17 +13680,16 @@
       <c r="E114" s="18" t="n">
         <v>46234.4259837963</v>
       </c>
-      <c r="F114" s="9">
-        <f>IF(OR(D114="",E114=""),"",(E114-D114)*24)</f>
-        <v/>
-      </c>
-      <c r="G114" s="9">
-        <f>IF(F114="","",F114/24)</f>
-        <v/>
-      </c>
-      <c r="H114" s="19">
-        <f>IF(D114="","",TEXT(D114,"YYYY-MM"))</f>
-        <v/>
+      <c r="F114" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G114" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H114" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="115">
@@ -13835,17 +13714,16 @@
       <c r="E115" s="18" t="n">
         <v>46234.4265162037</v>
       </c>
-      <c r="F115" s="9">
-        <f>IF(OR(D115="",E115=""),"",(E115-D115)*24)</f>
-        <v/>
-      </c>
-      <c r="G115" s="9">
-        <f>IF(F115="","",F115/24)</f>
-        <v/>
-      </c>
-      <c r="H115" s="19">
-        <f>IF(D115="","",TEXT(D115,"YYYY-MM"))</f>
-        <v/>
+      <c r="F115" s="9" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G115" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H115" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="116">
@@ -13866,17 +13744,16 @@
       <c r="E116" s="18" t="n">
         <v>46234.36974537037</v>
       </c>
-      <c r="F116" s="9">
-        <f>IF(OR(D116="",E116=""),"",(E116-D116)*24)</f>
-        <v/>
-      </c>
-      <c r="G116" s="9">
-        <f>IF(F116="","",F116/24)</f>
-        <v/>
-      </c>
-      <c r="H116" s="19">
-        <f>IF(D116="","",TEXT(D116,"YYYY-MM"))</f>
-        <v/>
+      <c r="F116" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G116" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="117">
@@ -13901,17 +13778,16 @@
       <c r="E117" s="18" t="n">
         <v>46234.51201388889</v>
       </c>
-      <c r="F117" s="9">
-        <f>IF(OR(D117="",E117=""),"",(E117-D117)*24)</f>
-        <v/>
-      </c>
-      <c r="G117" s="9">
-        <f>IF(F117="","",F117/24)</f>
-        <v/>
-      </c>
-      <c r="H117" s="19">
-        <f>IF(D117="","",TEXT(D117,"YYYY-MM"))</f>
-        <v/>
+      <c r="F117" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G117" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="118">
@@ -13936,17 +13812,16 @@
       <c r="E118" s="18" t="n">
         <v>46234.51248842593</v>
       </c>
-      <c r="F118" s="9">
-        <f>IF(OR(D118="",E118=""),"",(E118-D118)*24)</f>
-        <v/>
-      </c>
-      <c r="G118" s="9">
-        <f>IF(F118="","",F118/24)</f>
-        <v/>
-      </c>
-      <c r="H118" s="19">
-        <f>IF(D118="","",TEXT(D118,"YYYY-MM"))</f>
-        <v/>
+      <c r="F118" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G118" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="119">
@@ -13971,17 +13846,16 @@
       <c r="E119" s="18" t="n">
         <v>46234.58166666667</v>
       </c>
-      <c r="F119" s="9">
-        <f>IF(OR(D119="",E119=""),"",(E119-D119)*24)</f>
-        <v/>
-      </c>
-      <c r="G119" s="9">
-        <f>IF(F119="","",F119/24)</f>
-        <v/>
-      </c>
-      <c r="H119" s="19">
-        <f>IF(D119="","",TEXT(D119,"YYYY-MM"))</f>
-        <v/>
+      <c r="F119" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G119" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="120">
@@ -14006,17 +13880,16 @@
       <c r="E120" s="18" t="n">
         <v>46234.58244212963</v>
       </c>
-      <c r="F120" s="9">
-        <f>IF(OR(D120="",E120=""),"",(E120-D120)*24)</f>
-        <v/>
-      </c>
-      <c r="G120" s="9">
-        <f>IF(F120="","",F120/24)</f>
-        <v/>
-      </c>
-      <c r="H120" s="19">
-        <f>IF(D120="","",TEXT(D120,"YYYY-MM"))</f>
-        <v/>
+      <c r="F120" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G120" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="121">
@@ -14041,17 +13914,16 @@
       <c r="E121" s="18" t="n">
         <v>46234.58293981481</v>
       </c>
-      <c r="F121" s="9">
-        <f>IF(OR(D121="",E121=""),"",(E121-D121)*24)</f>
-        <v/>
-      </c>
-      <c r="G121" s="9">
-        <f>IF(F121="","",F121/24)</f>
-        <v/>
-      </c>
-      <c r="H121" s="19">
-        <f>IF(D121="","",TEXT(D121,"YYYY-MM"))</f>
-        <v/>
+      <c r="F121" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G121" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="122">
@@ -14076,17 +13948,16 @@
       <c r="E122" s="18" t="n">
         <v>46234.58412037037</v>
       </c>
-      <c r="F122" s="9">
-        <f>IF(OR(D122="",E122=""),"",(E122-D122)*24)</f>
-        <v/>
-      </c>
-      <c r="G122" s="9">
-        <f>IF(F122="","",F122/24)</f>
-        <v/>
-      </c>
-      <c r="H122" s="19">
-        <f>IF(D122="","",TEXT(D122,"YYYY-MM"))</f>
-        <v/>
+      <c r="F122" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G122" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" s="19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
       </c>
     </row>
     <row r="123">
@@ -14111,17 +13982,16 @@
       <c r="E123" s="18" t="n">
         <v>46245.38563657407</v>
       </c>
-      <c r="F123" s="9">
-        <f>IF(OR(D123="",E123=""),"",(E123-D123)*24)</f>
-        <v/>
-      </c>
-      <c r="G123" s="9">
-        <f>IF(F123="","",F123/24)</f>
-        <v/>
-      </c>
-      <c r="H123" s="19">
-        <f>IF(D123="","",TEXT(D123,"YYYY-MM"))</f>
-        <v/>
+      <c r="F123" s="9" t="n">
+        <v>190.2</v>
+      </c>
+      <c r="G123" s="9" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H123" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -14146,17 +14016,16 @@
       <c r="E124" s="18" t="n">
         <v>46245.38638888889</v>
       </c>
-      <c r="F124" s="9">
-        <f>IF(OR(D124="",E124=""),"",(E124-D124)*24)</f>
-        <v/>
-      </c>
-      <c r="G124" s="9">
-        <f>IF(F124="","",F124/24)</f>
-        <v/>
-      </c>
-      <c r="H124" s="19">
-        <f>IF(D124="","",TEXT(D124,"YYYY-MM"))</f>
-        <v/>
+      <c r="F124" s="9" t="n">
+        <v>190.1</v>
+      </c>
+      <c r="G124" s="9" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H124" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="125">
@@ -14181,17 +14050,16 @@
       <c r="E125" s="18" t="n">
         <v>46238.50366898148</v>
       </c>
-      <c r="F125" s="9">
-        <f>IF(OR(D125="",E125=""),"",(E125-D125)*24)</f>
-        <v/>
-      </c>
-      <c r="G125" s="9">
-        <f>IF(F125="","",F125/24)</f>
-        <v/>
-      </c>
-      <c r="H125" s="19">
-        <f>IF(D125="","",TEXT(D125,"YYYY-MM"))</f>
-        <v/>
+      <c r="F125" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G125" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="126">
@@ -14216,17 +14084,16 @@
       <c r="E126" s="18" t="n">
         <v>46238.50547453704</v>
       </c>
-      <c r="F126" s="9">
-        <f>IF(OR(D126="",E126=""),"",(E126-D126)*24)</f>
-        <v/>
-      </c>
-      <c r="G126" s="9">
-        <f>IF(F126="","",F126/24)</f>
-        <v/>
-      </c>
-      <c r="H126" s="19">
-        <f>IF(D126="","",TEXT(D126,"YYYY-MM"))</f>
-        <v/>
+      <c r="F126" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G126" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="127">
@@ -14251,17 +14118,16 @@
       <c r="E127" s="18" t="n">
         <v>46238.58211805556</v>
       </c>
-      <c r="F127" s="9">
-        <f>IF(OR(D127="",E127=""),"",(E127-D127)*24)</f>
-        <v/>
-      </c>
-      <c r="G127" s="9">
-        <f>IF(F127="","",F127/24)</f>
-        <v/>
-      </c>
-      <c r="H127" s="19">
-        <f>IF(D127="","",TEXT(D127,"YYYY-MM"))</f>
-        <v/>
+      <c r="F127" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G127" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="128">
@@ -14286,17 +14152,16 @@
       <c r="E128" s="18" t="n">
         <v>46245.38673611111</v>
       </c>
-      <c r="F128" s="9">
-        <f>IF(OR(D128="",E128=""),"",(E128-D128)*24)</f>
-        <v/>
-      </c>
-      <c r="G128" s="9">
-        <f>IF(F128="","",F128/24)</f>
-        <v/>
-      </c>
-      <c r="H128" s="19">
-        <f>IF(D128="","",TEXT(D128,"YYYY-MM"))</f>
-        <v/>
+      <c r="F128" s="9" t="n">
+        <v>162.2</v>
+      </c>
+      <c r="G128" s="9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H128" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="129">
@@ -14317,17 +14182,16 @@
       <c r="E129" s="18" t="n">
         <v>46239.45921296296</v>
       </c>
-      <c r="F129" s="9">
-        <f>IF(OR(D129="",E129=""),"",(E129-D129)*24)</f>
-        <v/>
-      </c>
-      <c r="G129" s="9">
-        <f>IF(F129="","",F129/24)</f>
-        <v/>
-      </c>
-      <c r="H129" s="19">
-        <f>IF(D129="","",TEXT(D129,"YYYY-MM"))</f>
-        <v/>
+      <c r="F129" s="9" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G129" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H129" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="130">
@@ -14352,17 +14216,16 @@
       <c r="E130" s="18" t="n">
         <v>46239.47231481481</v>
       </c>
-      <c r="F130" s="9">
-        <f>IF(OR(D130="",E130=""),"",(E130-D130)*24)</f>
-        <v/>
-      </c>
-      <c r="G130" s="9">
-        <f>IF(F130="","",F130/24)</f>
-        <v/>
-      </c>
-      <c r="H130" s="19">
-        <f>IF(D130="","",TEXT(D130,"YYYY-MM"))</f>
-        <v/>
+      <c r="F130" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G130" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="131">
@@ -14387,17 +14250,16 @@
       <c r="E131" s="18" t="n">
         <v>46240.38952546296</v>
       </c>
-      <c r="F131" s="9">
-        <f>IF(OR(D131="",E131=""),"",(E131-D131)*24)</f>
-        <v/>
-      </c>
-      <c r="G131" s="9">
-        <f>IF(F131="","",F131/24)</f>
-        <v/>
-      </c>
-      <c r="H131" s="19">
-        <f>IF(D131="","",TEXT(D131,"YYYY-MM"))</f>
-        <v/>
+      <c r="F131" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="132">
@@ -14422,17 +14284,16 @@
       <c r="E132" s="18" t="n">
         <v>46245.38721064815</v>
       </c>
-      <c r="F132" s="9">
-        <f>IF(OR(D132="",E132=""),"",(E132-D132)*24)</f>
-        <v/>
-      </c>
-      <c r="G132" s="9">
-        <f>IF(F132="","",F132/24)</f>
-        <v/>
-      </c>
-      <c r="H132" s="19">
-        <f>IF(D132="","",TEXT(D132,"YYYY-MM"))</f>
-        <v/>
+      <c r="F132" s="9" t="n">
+        <v>91.09999999999999</v>
+      </c>
+      <c r="G132" s="9" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="H132" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="133">
@@ -14457,17 +14318,16 @@
       <c r="E133" s="18" t="n">
         <v>46245.48166666667</v>
       </c>
-      <c r="F133" s="9">
-        <f>IF(OR(D133="",E133=""),"",(E133-D133)*24)</f>
-        <v/>
-      </c>
-      <c r="G133" s="9">
-        <f>IF(F133="","",F133/24)</f>
-        <v/>
-      </c>
-      <c r="H133" s="19">
-        <f>IF(D133="","",TEXT(D133,"YYYY-MM"))</f>
-        <v/>
+      <c r="F133" s="9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G133" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
     <row r="134">
@@ -14490,17 +14350,12 @@
         <v>46245.46525462963</v>
       </c>
       <c r="E134" s="18" t="n"/>
-      <c r="F134" s="9">
-        <f>IF(OR(D134="",E134=""),"",(E134-D134)*24)</f>
-        <v/>
-      </c>
-      <c r="G134" s="9">
-        <f>IF(F134="","",F134/24)</f>
-        <v/>
-      </c>
-      <c r="H134" s="19">
-        <f>IF(D134="","",TEXT(D134,"YYYY-MM"))</f>
-        <v/>
+      <c r="F134" s="9" t="n"/>
+      <c r="G134" s="9" t="n"/>
+      <c r="H134" s="19" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>